<commit_message>
Update Financial Workbook: tank stand full payment + June 27 balance
Tank stand entry moves from part payment (₦1,050,000) to full payment
(₦1,921,600). Stated balance line refreshed to 27/06/2026 figures
(₦2,181,100 in bank, ₦500,000 cash at hand, ₦2,681,100 grand total).
Report dates across sheets bumped to June 27, 2026.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NdiJob_Global_Financial_Workbook.xlsx
+++ b/NdiJob_Global_Financial_Workbook.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cover" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pledges" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Event Expenses" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gifts from Invitees" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Post-Event Expenses" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Balance Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pledges" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Expenses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gifts from Invitees" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Post-Event Expenses" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -317,7 +317,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -375,11 +375,128 @@
         <color rgb="000D1F3C"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000D1F3C"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="000D1F3C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000D1F3C"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="000D1F3C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000D1F3C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000D1F3C"/>
+      </right>
+      <top style="medium">
+        <color rgb="000D1F3C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000D1F3C"/>
+      </right>
+      <top style="medium">
+        <color rgb="000D1F3C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000D1F3C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000D1F3C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000D1F3C"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -665,6 +782,14 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1115,7 +1240,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Report Date: June 13, 2026</t>
+          <t>Report Date: June 27, 2026</t>
         </is>
       </c>
     </row>
@@ -1126,20 +1251,28 @@
           <t>OPENING ACCOUNT BALANCE</t>
         </is>
       </c>
+      <c r="C4" s="99" t="n"/>
+      <c r="D4" s="100" t="n"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>TOTAL PLEDGES (Job Family)</t>
         </is>
       </c>
+      <c r="G4" s="99" t="n"/>
+      <c r="H4" s="100" t="n"/>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="B5" s="5" t="n">
         <v>2950000</v>
       </c>
+      <c r="C5" s="101" t="n"/>
+      <c r="D5" s="102" t="n"/>
       <c r="F5" s="6">
         <f>Pledges!C17</f>
         <v/>
       </c>
+      <c r="G5" s="101" t="n"/>
+      <c r="H5" s="102" t="n"/>
     </row>
     <row r="6" ht="8" customHeight="1"/>
     <row r="7" ht="22" customHeight="1">
@@ -1148,21 +1281,29 @@
           <t>TOTAL EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="C7" s="99" t="n"/>
+      <c r="D7" s="100" t="n"/>
       <c r="F7" s="8" t="inlineStr">
         <is>
           <t>BALANCE AFTER EVENT</t>
         </is>
       </c>
+      <c r="G7" s="99" t="n"/>
+      <c r="H7" s="100" t="n"/>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="B8" s="9">
         <f>'Event Expenses'!D17</f>
         <v/>
       </c>
+      <c r="C8" s="101" t="n"/>
+      <c r="D8" s="102" t="n"/>
       <c r="F8" s="10">
         <f>'Event Expenses'!D18</f>
         <v/>
       </c>
+      <c r="G8" s="101" t="n"/>
+      <c r="H8" s="102" t="n"/>
     </row>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="22" customHeight="1">
@@ -1171,21 +1312,29 @@
           <t>TOTAL GIFTS RECEIVED</t>
         </is>
       </c>
+      <c r="C10" s="99" t="n"/>
+      <c r="D10" s="100" t="n"/>
       <c r="F10" s="12" t="inlineStr">
         <is>
           <t>GROSS TOTAL (before post-exp)</t>
         </is>
       </c>
+      <c r="G10" s="99" t="n"/>
+      <c r="H10" s="100" t="n"/>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="B11" s="13">
         <f>'Gifts from Invitees'!C21</f>
         <v/>
       </c>
+      <c r="C11" s="101" t="n"/>
+      <c r="D11" s="102" t="n"/>
       <c r="F11" s="14">
         <f>'Gifts from Invitees'!C22</f>
         <v/>
       </c>
+      <c r="G11" s="101" t="n"/>
+      <c r="H11" s="102" t="n"/>
     </row>
     <row r="12" ht="8" customHeight="1"/>
     <row r="13" ht="22" customHeight="1">
@@ -1194,21 +1343,29 @@
           <t>TOTAL POST-EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="C13" s="99" t="n"/>
+      <c r="D13" s="100" t="n"/>
       <c r="F13" s="16" t="inlineStr">
         <is>
           <t>NET FINAL BALANCE</t>
         </is>
       </c>
+      <c r="G13" s="99" t="n"/>
+      <c r="H13" s="100" t="n"/>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="B14" s="17">
         <f>'Post-Event Expenses'!C7</f>
         <v/>
       </c>
+      <c r="C14" s="101" t="n"/>
+      <c r="D14" s="102" t="n"/>
       <c r="F14" s="18">
         <f>'Balance Summary'!D50</f>
         <v/>
       </c>
+      <c r="G14" s="101" t="n"/>
+      <c r="H14" s="102" t="n"/>
     </row>
     <row r="15" ht="14" customHeight="1"/>
     <row r="16" ht="22" customHeight="1">
@@ -1217,6 +1374,8 @@
           <t>EVENT EXPENSE BREAKDOWN</t>
         </is>
       </c>
+      <c r="C16" s="103" t="n"/>
+      <c r="D16" s="104" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="20" t="inlineStr">
@@ -1406,6 +1565,8 @@
           <t>GIFTS FROM INVITEES</t>
         </is>
       </c>
+      <c r="C31" s="103" t="n"/>
+      <c r="D31" s="104" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="20" t="inlineStr">
@@ -1644,6 +1805,15 @@
           <t>DISCLAIMER: This document is confidential and intended solely for authorised recipients of NDIJOB GLOBAL.</t>
         </is>
       </c>
+      <c r="B50" s="103" t="n"/>
+      <c r="C50" s="103" t="n"/>
+      <c r="D50" s="103" t="n"/>
+      <c r="E50" s="103" t="n"/>
+      <c r="F50" s="103" t="n"/>
+      <c r="G50" s="103" t="n"/>
+      <c r="H50" s="103" t="n"/>
+      <c r="I50" s="103" t="n"/>
+      <c r="J50" s="104" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -1709,7 +1879,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated: June 13, 2026  |  All figures in Nigerian Naira (₦)</t>
+          <t>Generated: June 27, 2026  |  All figures in Nigerian Naira (₦)</t>
         </is>
       </c>
     </row>
@@ -1720,11 +1890,15 @@
           <t>CONTENTS</t>
         </is>
       </c>
+      <c r="B5" s="104" t="n"/>
       <c r="C5" s="32" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
+      <c r="D5" s="103" t="n"/>
+      <c r="E5" s="103" t="n"/>
+      <c r="F5" s="104" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="33" t="inlineStr">
@@ -1732,11 +1906,15 @@
           <t>Pledges</t>
         </is>
       </c>
+      <c r="B6" s="104" t="n"/>
       <c r="C6" s="34" t="inlineStr">
         <is>
           <t>Job Family contributions &amp; payments</t>
         </is>
       </c>
+      <c r="D6" s="103" t="n"/>
+      <c r="E6" s="103" t="n"/>
+      <c r="F6" s="104" t="n"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="35" t="inlineStr">
@@ -1744,11 +1922,15 @@
           <t>Event Expenses</t>
         </is>
       </c>
+      <c r="B7" s="104" t="n"/>
       <c r="C7" s="36" t="inlineStr">
         <is>
           <t>All expenses incurred for the event</t>
         </is>
       </c>
+      <c r="D7" s="103" t="n"/>
+      <c r="E7" s="103" t="n"/>
+      <c r="F7" s="104" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="37" t="inlineStr">
@@ -1756,11 +1938,15 @@
           <t>Gifts</t>
         </is>
       </c>
+      <c r="B8" s="104" t="n"/>
       <c r="C8" s="38" t="inlineStr">
         <is>
           <t>Donations received from event invitees</t>
         </is>
       </c>
+      <c r="D8" s="103" t="n"/>
+      <c r="E8" s="103" t="n"/>
+      <c r="F8" s="104" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="39" t="inlineStr">
@@ -1768,11 +1954,15 @@
           <t>Post-Event Exp.</t>
         </is>
       </c>
+      <c r="B9" s="104" t="n"/>
       <c r="C9" s="40" t="inlineStr">
         <is>
           <t>Infrastructure &amp; operational spending</t>
         </is>
       </c>
+      <c r="D9" s="103" t="n"/>
+      <c r="E9" s="103" t="n"/>
+      <c r="F9" s="104" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="41" t="inlineStr">
@@ -1780,11 +1970,15 @@
           <t>Balance Summary</t>
         </is>
       </c>
+      <c r="B10" s="104" t="n"/>
       <c r="C10" s="42" t="inlineStr">
         <is>
           <t>Full running statement with net balance</t>
         </is>
       </c>
+      <c r="D10" s="103" t="n"/>
+      <c r="E10" s="103" t="n"/>
+      <c r="F10" s="104" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="43" t="inlineStr">
@@ -1792,11 +1986,15 @@
           <t>Dashboard</t>
         </is>
       </c>
+      <c r="B11" s="104" t="n"/>
       <c r="C11" s="44" t="inlineStr">
         <is>
           <t>Visual summary of all key figures</t>
         </is>
       </c>
+      <c r="D11" s="103" t="n"/>
+      <c r="E11" s="103" t="n"/>
+      <c r="F11" s="104" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -1805,12 +2003,12 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C8:F8"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="C7:F7"/>
-    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A9:B9"/>
     <mergeCell ref="C11:F11"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C5:F5"/>
@@ -1851,7 +2049,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="46" t="inlineStr">
         <is>
-          <t>All amounts in Nigerian Naira (₦)  |  Generated: June 13, 2026</t>
+          <t>All amounts in Nigerian Naira (₦)  |  Generated: June 27, 2026</t>
         </is>
       </c>
     </row>
@@ -2275,6 +2473,7 @@
           <t>TOTAL PLEDGES / PAYMENTS</t>
         </is>
       </c>
+      <c r="B17" s="105" t="n"/>
       <c r="C17" s="59">
         <f>SUM(C4:C16)</f>
         <v/>
@@ -2296,6 +2495,12 @@
           <t xml:space="preserve">  ★  Money deposited in account: ₦2,950,000</t>
         </is>
       </c>
+      <c r="B18" s="103" t="n"/>
+      <c r="C18" s="103" t="n"/>
+      <c r="D18" s="103" t="n"/>
+      <c r="E18" s="103" t="n"/>
+      <c r="F18" s="103" t="n"/>
+      <c r="G18" s="104" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2339,7 +2544,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="46" t="inlineStr">
         <is>
-          <t>All amounts in Nigerian Naira (₦)  |  Generated: June 13, 2026</t>
+          <t>All amounts in Nigerian Naira (₦)  |  Generated: June 27, 2026</t>
         </is>
       </c>
     </row>
@@ -2693,6 +2898,8 @@
           <t>TOTAL EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="B17" s="106" t="n"/>
+      <c r="C17" s="105" t="n"/>
       <c r="D17" s="60">
         <f>SUM(D4:D16)</f>
         <v/>
@@ -2706,6 +2913,8 @@
           <t>BALANCE AFTER EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="B18" s="106" t="n"/>
+      <c r="C18" s="105" t="n"/>
       <c r="D18" s="66">
         <f>2950000-D17</f>
         <v/>
@@ -2719,6 +2928,11 @@
           <t xml:space="preserve">  ★  Stated balance per records: ₦986,600</t>
         </is>
       </c>
+      <c r="B19" s="103" t="n"/>
+      <c r="C19" s="103" t="n"/>
+      <c r="D19" s="103" t="n"/>
+      <c r="E19" s="103" t="n"/>
+      <c r="F19" s="104" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2762,7 +2976,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="46" t="inlineStr">
         <is>
-          <t>All amounts in Nigerian Naira (₦)  |  Generated: June 13, 2026</t>
+          <t>All amounts in Nigerian Naira (₦)  |  Generated: June 27, 2026</t>
         </is>
       </c>
     </row>
@@ -2772,6 +2986,8 @@
           <t>Balance B/F (after event expenses)</t>
         </is>
       </c>
+      <c r="B3" s="106" t="n"/>
+      <c r="C3" s="105" t="n"/>
       <c r="D3" s="68" t="n">
         <v>986600</v>
       </c>
@@ -3154,6 +3370,7 @@
           <t>TOTAL GIFTS RECEIVED</t>
         </is>
       </c>
+      <c r="B21" s="105" t="n"/>
       <c r="C21" s="59">
         <f>SUM(C5:C20)</f>
         <v/>
@@ -3167,6 +3384,7 @@
           <t>GRAND TOTAL  (B/F + Gifts)</t>
         </is>
       </c>
+      <c r="B22" s="105" t="n"/>
       <c r="C22" s="71">
         <f>986600+C21</f>
         <v/>
@@ -3216,7 +3434,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="46" t="inlineStr">
         <is>
-          <t>Infrastructure &amp; operational expenditure  |  Generated: June 13, 2026</t>
+          <t>Infrastructure &amp; operational expenditure  |  Generated: June 27, 2026</t>
         </is>
       </c>
     </row>
@@ -3253,11 +3471,11 @@
       </c>
       <c r="B4" s="49" t="inlineStr">
         <is>
-          <t>Part Payment – Tank Stand</t>
+          <t>Full Payment – Tank Stand</t>
         </is>
       </c>
       <c r="C4" s="50" t="n">
-        <v>1050000</v>
+        <v>1921600</v>
       </c>
       <c r="D4" s="49" t="inlineStr"/>
       <c r="E4" s="49" t="inlineStr"/>
@@ -3298,6 +3516,7 @@
           <t>TOTAL POST-EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="B7" s="105" t="n"/>
       <c r="C7" s="60">
         <f>SUM(C4:C6)</f>
         <v/>
@@ -3344,7 +3563,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="46" t="inlineStr">
         <is>
-          <t>As at June 13, 2026</t>
+          <t>As at June 27, 2026</t>
         </is>
       </c>
     </row>
@@ -3354,6 +3573,7 @@
           <t>Item</t>
         </is>
       </c>
+      <c r="B3" s="105" t="n"/>
       <c r="C3" s="74" t="inlineStr">
         <is>
           <t>Amount (₦)</t>
@@ -3371,6 +3591,9 @@
           <t>A.  OPENING — JOB FAMILY CONTRIBUTIONS</t>
         </is>
       </c>
+      <c r="B4" s="106" t="n"/>
+      <c r="C4" s="106" t="n"/>
+      <c r="D4" s="105" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="76" t="inlineStr">
@@ -3378,6 +3601,7 @@
           <t xml:space="preserve">    Money deposited in account</t>
         </is>
       </c>
+      <c r="B5" s="104" t="n"/>
       <c r="C5" s="77" t="n">
         <v>2950000</v>
       </c>
@@ -3397,6 +3621,9 @@
           <t>B.  EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="B7" s="106" t="n"/>
+      <c r="C7" s="106" t="n"/>
+      <c r="D7" s="105" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="76" t="inlineStr">
@@ -3404,6 +3631,7 @@
           <t xml:space="preserve">      1. DJ</t>
         </is>
       </c>
+      <c r="B8" s="104" t="n"/>
       <c r="C8" s="77" t="n">
         <v>120000</v>
       </c>
@@ -3415,6 +3643,7 @@
           <t xml:space="preserve">      2. Advert</t>
         </is>
       </c>
+      <c r="B9" s="104" t="n"/>
       <c r="C9" s="77" t="n">
         <v>120000</v>
       </c>
@@ -3426,6 +3655,7 @@
           <t xml:space="preserve">      3. Caterer</t>
         </is>
       </c>
+      <c r="B10" s="104" t="n"/>
       <c r="C10" s="77" t="n">
         <v>430000</v>
       </c>
@@ -3437,6 +3667,7 @@
           <t xml:space="preserve">      4. Canopies, Tables &amp; Chairs</t>
         </is>
       </c>
+      <c r="B11" s="104" t="n"/>
       <c r="C11" s="77" t="n">
         <v>150000</v>
       </c>
@@ -3448,6 +3679,7 @@
           <t xml:space="preserve">      5. Registration of Name</t>
         </is>
       </c>
+      <c r="B12" s="104" t="n"/>
       <c r="C12" s="77" t="n">
         <v>42000</v>
       </c>
@@ -3459,6 +3691,7 @@
           <t xml:space="preserve">      6. Decorations</t>
         </is>
       </c>
+      <c r="B13" s="104" t="n"/>
       <c r="C13" s="77" t="n">
         <v>110000</v>
       </c>
@@ -3470,6 +3703,7 @@
           <t xml:space="preserve">      7. Drinks / Water</t>
         </is>
       </c>
+      <c r="B14" s="104" t="n"/>
       <c r="C14" s="77" t="n">
         <v>348400</v>
       </c>
@@ -3481,6 +3715,7 @@
           <t xml:space="preserve">      8. XXXXLT-Shirts</t>
         </is>
       </c>
+      <c r="B15" s="104" t="n"/>
       <c r="C15" s="77" t="n">
         <v>48000</v>
       </c>
@@ -3492,6 +3727,7 @@
           <t xml:space="preserve">      9. Meat / Garden Egg / Kolanut</t>
         </is>
       </c>
+      <c r="B16" s="104" t="n"/>
       <c r="C16" s="77" t="n">
         <v>525000</v>
       </c>
@@ -3503,6 +3739,7 @@
           <t xml:space="preserve">      10. Firewood</t>
         </is>
       </c>
+      <c r="B17" s="104" t="n"/>
       <c r="C17" s="77" t="n">
         <v>30000</v>
       </c>
@@ -3514,6 +3751,7 @@
           <t xml:space="preserve">      11. MC</t>
         </is>
       </c>
+      <c r="B18" s="104" t="n"/>
       <c r="C18" s="77" t="n">
         <v>130000</v>
       </c>
@@ -3525,6 +3763,7 @@
           <t xml:space="preserve">      12. Ice Block</t>
         </is>
       </c>
+      <c r="B19" s="104" t="n"/>
       <c r="C19" s="77" t="n">
         <v>12000</v>
       </c>
@@ -3536,6 +3775,7 @@
           <t xml:space="preserve">      13. Shehu (Cash)</t>
         </is>
       </c>
+      <c r="B20" s="104" t="n"/>
       <c r="C20" s="77" t="n">
         <v>8000</v>
       </c>
@@ -3547,6 +3787,7 @@
           <t>TOTAL EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="B21" s="104" t="n"/>
       <c r="C21" s="83">
         <f>SUM(C8:C20)</f>
         <v/>
@@ -3562,6 +3803,9 @@
           <t xml:space="preserve">  ★  Stated balance after event expenses: ₦986,600</t>
         </is>
       </c>
+      <c r="B22" s="103" t="n"/>
+      <c r="C22" s="103" t="n"/>
+      <c r="D22" s="104" t="n"/>
     </row>
     <row r="23" ht="8" customHeight="1">
       <c r="A23" s="79" t="n"/>
@@ -3575,6 +3819,9 @@
           <t>C.  GIFTS FROM INVITEES</t>
         </is>
       </c>
+      <c r="B24" s="106" t="n"/>
+      <c r="C24" s="106" t="n"/>
+      <c r="D24" s="105" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="76" t="inlineStr">
@@ -3582,6 +3829,7 @@
           <t xml:space="preserve">      1. Nkechi Umunakwe</t>
         </is>
       </c>
+      <c r="B25" s="104" t="n"/>
       <c r="C25" s="77" t="n">
         <v>150000</v>
       </c>
@@ -3593,6 +3841,7 @@
           <t xml:space="preserve">      2. Casmir Chimankpam Ebelleme</t>
         </is>
       </c>
+      <c r="B26" s="104" t="n"/>
       <c r="C26" s="77" t="n">
         <v>20000</v>
       </c>
@@ -3604,6 +3853,7 @@
           <t xml:space="preserve">      3. Max</t>
         </is>
       </c>
+      <c r="B27" s="104" t="n"/>
       <c r="C27" s="77" t="n">
         <v>100000</v>
       </c>
@@ -3615,6 +3865,7 @@
           <t xml:space="preserve">      4. Prof BEB Nwoke</t>
         </is>
       </c>
+      <c r="B28" s="104" t="n"/>
       <c r="C28" s="77" t="n">
         <v>100000</v>
       </c>
@@ -3626,6 +3877,7 @@
           <t xml:space="preserve">      5. Benedict</t>
         </is>
       </c>
+      <c r="B29" s="104" t="n"/>
       <c r="C29" s="77" t="n">
         <v>1000000</v>
       </c>
@@ -3637,6 +3889,7 @@
           <t xml:space="preserve">      6. Chibuzor</t>
         </is>
       </c>
+      <c r="B30" s="104" t="n"/>
       <c r="C30" s="77" t="n">
         <v>50000</v>
       </c>
@@ -3648,6 +3901,7 @@
           <t xml:space="preserve">      7. Odoh Chike Nnaemeka</t>
         </is>
       </c>
+      <c r="B31" s="104" t="n"/>
       <c r="C31" s="77" t="n">
         <v>100000</v>
       </c>
@@ -3659,6 +3913,7 @@
           <t xml:space="preserve">      8. Odoh Chike Nnaemeka</t>
         </is>
       </c>
+      <c r="B32" s="104" t="n"/>
       <c r="C32" s="77" t="n">
         <v>21000</v>
       </c>
@@ -3670,6 +3925,7 @@
           <t xml:space="preserve">      9. Cash – Day of Event</t>
         </is>
       </c>
+      <c r="B33" s="104" t="n"/>
       <c r="C33" s="77" t="n">
         <v>153000</v>
       </c>
@@ -3681,6 +3937,7 @@
           <t xml:space="preserve">      10. Emma Obinikpa</t>
         </is>
       </c>
+      <c r="B34" s="104" t="n"/>
       <c r="C34" s="77" t="n">
         <v>100000</v>
       </c>
@@ -3692,6 +3949,7 @@
           <t xml:space="preserve">      11. Odoh Chike Nnamdi</t>
         </is>
       </c>
+      <c r="B35" s="104" t="n"/>
       <c r="C35" s="77" t="n">
         <v>500000</v>
       </c>
@@ -3703,6 +3961,7 @@
           <t xml:space="preserve">      12. Mrs Pearl Kanu</t>
         </is>
       </c>
+      <c r="B36" s="104" t="n"/>
       <c r="C36" s="77" t="n">
         <v>200000</v>
       </c>
@@ -3714,6 +3973,7 @@
           <t xml:space="preserve">      13. Mrs Ibekwe</t>
         </is>
       </c>
+      <c r="B37" s="104" t="n"/>
       <c r="C37" s="77" t="n">
         <v>500000</v>
       </c>
@@ -3725,6 +3985,7 @@
           <t xml:space="preserve">      14. Favour Njoku</t>
         </is>
       </c>
+      <c r="B38" s="104" t="n"/>
       <c r="C38" s="77" t="n">
         <v>100000</v>
       </c>
@@ -3736,6 +3997,7 @@
           <t xml:space="preserve">      15. Ify Ohameje</t>
         </is>
       </c>
+      <c r="B39" s="104" t="n"/>
       <c r="C39" s="77" t="n">
         <v>200000</v>
       </c>
@@ -3747,6 +4009,7 @@
           <t xml:space="preserve">      16. Dubem Nnayere Odoh</t>
         </is>
       </c>
+      <c r="B40" s="104" t="n"/>
       <c r="C40" s="77" t="n">
         <v>400000</v>
       </c>
@@ -3758,6 +4021,7 @@
           <t>TOTAL GIFTS RECEIVED</t>
         </is>
       </c>
+      <c r="B41" s="104" t="n"/>
       <c r="C41" s="88">
         <f>SUM(C25:C40)</f>
         <v/>
@@ -3773,6 +4037,7 @@
           <t>GROSS TOTAL AVAILABLE  (29/12/2025)</t>
         </is>
       </c>
+      <c r="B42" s="105" t="n"/>
       <c r="C42" s="61" t="n"/>
       <c r="D42" s="91">
         <f>D41</f>
@@ -3791,15 +4056,19 @@
           <t>D.  POST-EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="B44" s="106" t="n"/>
+      <c r="C44" s="106" t="n"/>
+      <c r="D44" s="105" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">      1. Part Payment – Tank Stand</t>
-        </is>
-      </c>
+          <t xml:space="preserve">      1. Full Payment – Tank Stand</t>
+        </is>
+      </c>
+      <c r="B45" s="104" t="n"/>
       <c r="C45" s="77" t="n">
-        <v>1050000</v>
+        <v>1921600</v>
       </c>
       <c r="D45" s="81" t="n"/>
     </row>
@@ -3809,6 +4078,7 @@
           <t xml:space="preserve">      2. Cutting of Grass</t>
         </is>
       </c>
+      <c r="B46" s="104" t="n"/>
       <c r="C46" s="77" t="n">
         <v>20000</v>
       </c>
@@ -3820,6 +4090,7 @@
           <t xml:space="preserve">      3. First Instalment – Borehole</t>
         </is>
       </c>
+      <c r="B47" s="104" t="n"/>
       <c r="C47" s="77" t="n">
         <v>2759500</v>
       </c>
@@ -3831,6 +4102,7 @@
           <t>TOTAL POST-EVENT EXPENSES</t>
         </is>
       </c>
+      <c r="B48" s="104" t="n"/>
       <c r="C48" s="94">
         <f>SUM(C45:C47)</f>
         <v/>
@@ -3849,6 +4121,7 @@
           <t>★  NET FINAL BALANCE</t>
         </is>
       </c>
+      <c r="B50" s="105" t="n"/>
       <c r="C50" s="61" t="n"/>
       <c r="D50" s="97">
         <f>D42-C48</f>
@@ -3858,9 +4131,12 @@
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="98" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ★  Stated balance per records (29/12/2025): ₦2,350,560</t>
-        </is>
-      </c>
+          <t xml:space="preserve">  ★  Stated balance per records (27/06/2026): ₦2,181,100  |  Cash at hand 2026: ₦500,000  |  Grand total: ₦2,681,100</t>
+        </is>
+      </c>
+      <c r="B51" s="103" t="n"/>
+      <c r="C51" s="103" t="n"/>
+      <c r="D51" s="104" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="47">

</xml_diff>